<commit_message>
Plan to design cpu (add opcode)
</commit_message>
<xml_diff>
--- a/document/SoC_Design.xlsx
+++ b/document/SoC_Design.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CB5E53-332E-4C94-B75D-4634808A13A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF24DEBF-CF2A-41EB-92C9-AF05ADD4482E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="18615" windowHeight="15585" activeTab="4" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
   <sheets>
     <sheet name="TASK" sheetId="1" r:id="rId1"/>
     <sheet name="오류사항분석" sheetId="2" r:id="rId2"/>
     <sheet name="MemoryMap" sheetId="4" r:id="rId3"/>
     <sheet name="교안참고" sheetId="3" r:id="rId4"/>
+    <sheet name="미구현명령어 정리" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="112">
   <si>
     <t>No</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -335,6 +336,162 @@
   </si>
   <si>
     <t>CACHE MEMORY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>명령어</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>구분방법</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bgezal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b000001 (REGIMM), rt = 5'b1001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bltz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bgez</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bltzal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b000001 (REGIMM), rt = 5'b0000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b000001 (REGIMM), rt = 5'b0001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b000001 (REGIMM), rt = 5'b1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Branch on Greater Than or Equal to Zero (&gt;= 0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Branch on Less Than Zero (&lt; 0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Branch on Less Than Zero (&lt; 0) And Link ($ra &lt;= PC)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Branch on Greater Than or Equal to Zero (&gt;= 0) And Link ($ra &lt;= PC)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jalr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jump and Link Register</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b000000, funct_code = 6'b0001001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>verilogHDL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정의(동작)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>구현 유무</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lbu</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lb</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load Byte Unsigned (opcode-rs-rt-imm &lt;=&gt; lbu rt, imm(rs)) (zero-extend)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load Byte (opcode-rs-rt-imm &lt;=&gt; lb rt, imm(rs)) (sign-extend)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b100000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b100100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lhu</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sb</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load Half-Word Unsigned (opcode-rs-rt-imm &lt;=&gt; lhu rt, imm(rs)) (zero-extend)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load Half-Word (opcode-rs-rt-imm &lt;=&gt; lh rt, imm(rs)) (sign-extend)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b100001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>opcode = 6'b100101</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stroe Half-Word (opcode-rs-rt-imm &lt;=&gt; sh rt, imm(rs))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Store Byte (opcode-rs-rt-imm &lt;=&gt; sb rt, imm(rs))</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1810,4 +1967,292 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA67579D-FAA6-4F15-B946-E6672032C149}">
+  <dimension ref="B2:G14"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="76.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="G2" s="12"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <f>B4+1</f>
+        <v>2</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <f>B5+1</f>
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
+        <f>B6+1</f>
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B8" s="1">
+        <f>B7+1</f>
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <f>B8+1</f>
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="1">
+        <f>B9+1</f>
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <f>B10+1</f>
+        <v>8</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <f>B11+1</f>
+        <v>9</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <f>B12+1</f>
+        <v>10</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <f>B13+1</f>
+        <v>11</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:G2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>